<commit_message>
finalizando a parte do cadastro e acesso as planilhas
</commit_message>
<xml_diff>
--- a/Site More Speed/docs/cadastros.xlsx
+++ b/Site More Speed/docs/cadastros.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="9">
   <si>
     <t>Clientes Cadastrados</t>
   </si>
@@ -42,9 +42,6 @@
   </si>
   <si>
     <t>MORE10</t>
-  </si>
-  <si>
-    <t>Carlos Eduardo</t>
   </si>
 </sst>
 </file>
@@ -405,7 +402,7 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:D3"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="35" customWidth="true" style="0"/>
@@ -447,20 +444,6 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:4">
-      <c r="A4" t="s">
-        <v>9</v>
-      </c>
-      <c r="B4" t="s">
-        <v>6</v>
-      </c>
-      <c r="C4" t="s">
-        <v>7</v>
-      </c>
-      <c r="D4" t="s">
-        <v>8</v>
-      </c>
-    </row>
   </sheetData>
   <mergeCells>
     <mergeCell ref="A1:D1"/>

</xml_diff>